<commit_message>
Group EX HITACHI 1797 summary by product type (diodes / thyristors) with subtotals
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3tLabRpvRXjmQSLze128h
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Hitachi_Shindengen_EX1797.xlsx
+++ b/output/HS_Code_Summary_Hitachi_Shindengen_EX1797.xlsx
@@ -44,7 +44,7 @@
     </font>
     <font/>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -58,7 +58,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EAF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -98,24 +108,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -135,6 +138,27 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -504,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -613,543 +637,639 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
+          <t>DIODES  —  HS 8541 10 00</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
           <t>Diode</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>5SDD 24F2800</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>5SDD 24F2800 Rectifier diodes</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>85411000</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E7" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F7" s="9" t="n">
         <v>19.6</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G7" s="9" t="n">
         <v>21.6</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H7" s="9" t="n">
         <v>168</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="I7" s="9" t="n">
         <v>6720</v>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="J7" s="10" t="inlineStr">
         <is>
           <t>810678828</t>
         </is>
       </c>
-      <c r="K6" s="8" t="inlineStr">
+      <c r="K7" s="10" t="inlineStr">
         <is>
           <t>0923633858</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="L7" s="7" t="inlineStr">
         <is>
           <t>FCA Prague</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M7" s="7" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Diode</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>5SDA 14F5007</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>5SDA 14F5007 Avalanche diodes</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>85411000</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E8" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F8" s="9" t="n">
         <v>2.35</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G8" s="9" t="n">
         <v>2.6</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H8" s="9" t="n">
         <v>209</v>
       </c>
-      <c r="I7" s="7" t="n">
+      <c r="I8" s="9" t="n">
         <v>1045</v>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="J8" s="10" t="inlineStr">
         <is>
           <t>810678829</t>
         </is>
       </c>
-      <c r="K7" s="8" t="inlineStr">
+      <c r="K8" s="10" t="inlineStr">
         <is>
           <t>0923633901</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="L8" s="7" t="inlineStr">
         <is>
           <t>FCA Prague</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="M8" s="7" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Thyristor</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>5STP 3328L0011</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>YST 45 P28 E / Thyristor</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>85413000</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>140</v>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>140</v>
-      </c>
-      <c r="H8" s="12" t="n">
-        <v>484</v>
-      </c>
-      <c r="I8" s="12" t="n">
-        <v>48400</v>
-      </c>
-      <c r="J8" s="13" t="inlineStr">
-        <is>
-          <t>810678830</t>
-        </is>
-      </c>
-      <c r="K8" s="13" t="inlineStr">
-        <is>
-          <t>0923633955</t>
-        </is>
-      </c>
-      <c r="L8" s="10" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Diode</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>5SDD 3050L0003</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>YSD 45-02 P50 / Diode</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>85411000</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>58.75</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>58.75</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>549</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>25803</v>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>810678834</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>0923634051</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
         <is>
           <t>FCA Prague</t>
         </is>
       </c>
-      <c r="M8" s="10" t="inlineStr">
+      <c r="M9" s="7" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Thyristor</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>5STP 12F4200</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>YST 14-29 P42D / Thyristor</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>85413000</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="F9" s="12" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="G9" s="12" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="H9" s="12" t="n">
-        <v>181</v>
-      </c>
-      <c r="I9" s="12" t="n">
-        <v>905</v>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
-        <is>
-          <t>810678833</t>
-        </is>
-      </c>
-      <c r="K9" s="13" t="inlineStr">
-        <is>
-          <t>0923633974</t>
-        </is>
-      </c>
-      <c r="L9" s="10" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Diode</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>5SDD7102B0001</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>5SDD 7102B0001 Welding diodes</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>85411000</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>28400</v>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>810678853</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>0923637756</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>FCA Prague</t>
         </is>
       </c>
-      <c r="M9" s="10" t="inlineStr">
+      <c r="M10" s="7" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Diode</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>5SDD 3050L0003</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>YSD 45-02 P50 / Diode</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>5SDD0135Z0401</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>5SDD 0135Z0401 Welding diodes</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>85411000</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n">
-        <v>47</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>58.75</v>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>58.75</v>
-      </c>
-      <c r="H10" s="7" t="n">
-        <v>549</v>
-      </c>
-      <c r="I10" s="7" t="n">
-        <v>25803</v>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>810678834</t>
-        </is>
-      </c>
-      <c r="K10" s="8" t="inlineStr">
-        <is>
-          <t>0923634051</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
+      <c r="E11" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>108</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>21600</v>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>810678854</t>
+        </is>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>0923637801</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
         <is>
           <t>FCA Prague</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M11" s="7" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Thyristor</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>5STP2552L0025</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>PCT 5200 V 2500 A SF Thyristor</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>85413000</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>60</v>
-      </c>
-      <c r="F11" s="12" t="n">
-        <v>87</v>
-      </c>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="n">
-        <v>442</v>
-      </c>
-      <c r="I11" s="12" t="n">
-        <v>26520</v>
-      </c>
-      <c r="J11" s="13" t="inlineStr">
-        <is>
-          <t>810678838</t>
-        </is>
-      </c>
-      <c r="K11" s="13" t="inlineStr">
-        <is>
-          <t>0923634362</t>
-        </is>
-      </c>
-      <c r="L11" s="10" t="inlineStr">
-        <is>
-          <t>FCA Prague</t>
-        </is>
-      </c>
-      <c r="M11" s="10" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-    </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Diode</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>5SDD7102B0001</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>5SDD 7102B0001 Welding diodes</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>85411000</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>56</v>
-      </c>
-      <c r="G12" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="H12" s="7" t="n">
-        <v>71</v>
-      </c>
-      <c r="I12" s="7" t="n">
-        <v>28400</v>
-      </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>810678853</t>
-        </is>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>0923637756</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>FCA Prague</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal — DIODES  —  HS 8541 10 00 (5 items)</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="13" t="n">
+        <v>692</v>
+      </c>
+      <c r="F12" s="14" t="n">
+        <v>164.7</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>176.95</v>
+      </c>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="14" t="n">
+        <v>83568</v>
+      </c>
+      <c r="J12" s="11" t="n"/>
+      <c r="K12" s="11" t="n"/>
+      <c r="L12" s="12" t="n"/>
+      <c r="M12" s="12" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Diode</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>5SDD0135Z0401</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>5SDD 0135Z0401 Welding diodes</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>85411000</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>200</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="G13" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>108</v>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>21600</v>
-      </c>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>810678854</t>
-        </is>
-      </c>
-      <c r="K13" s="8" t="inlineStr">
-        <is>
-          <t>0923637801</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
+          <t>THYRISTORS  —  HS 8541 30 00</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
+      <c r="M13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Thyristor</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>5STP 3328L0011</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>YST 45 P28 E / Thyristor</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>85413000</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>100</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>140</v>
+      </c>
+      <c r="G14" s="18" t="n">
+        <v>140</v>
+      </c>
+      <c r="H14" s="18" t="n">
+        <v>484</v>
+      </c>
+      <c r="I14" s="18" t="n">
+        <v>48400</v>
+      </c>
+      <c r="J14" s="19" t="inlineStr">
+        <is>
+          <t>810678830</t>
+        </is>
+      </c>
+      <c r="K14" s="19" t="inlineStr">
+        <is>
+          <t>0923633955</t>
+        </is>
+      </c>
+      <c r="L14" s="16" t="inlineStr">
         <is>
           <t>FCA Prague</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M14" s="16" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="14" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Thyristor</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>5STP 12F4200</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>YST 14-29 P42D / Thyristor</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>85413000</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="18" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G15" s="18" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="H15" s="18" t="n">
+        <v>181</v>
+      </c>
+      <c r="I15" s="18" t="n">
+        <v>905</v>
+      </c>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>810678833</t>
+        </is>
+      </c>
+      <c r="K15" s="19" t="inlineStr">
+        <is>
+          <t>0923633974</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>FCA Prague</t>
+        </is>
+      </c>
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Thyristor</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>5STP2552L0025</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>PCT 5200 V 2500 A SF Thyristor</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>85413000</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>60</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>87</v>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>442</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>26520</v>
+      </c>
+      <c r="J16" s="19" t="inlineStr">
+        <is>
+          <t>810678838</t>
+        </is>
+      </c>
+      <c r="K16" s="19" t="inlineStr">
+        <is>
+          <t>0923634362</t>
+        </is>
+      </c>
+      <c r="L16" s="16" t="inlineStr">
+        <is>
+          <t>FCA Prague</t>
+        </is>
+      </c>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal — THYRISTORS  —  HS 8541 30 00 (3 items)</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="13" t="n">
+        <v>165</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>229.4</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>142.75</v>
+      </c>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="14" t="n">
+        <v>75825</v>
+      </c>
+      <c r="J17" s="11" t="n"/>
+      <c r="K17" s="11" t="n"/>
+      <c r="L17" s="12" t="n"/>
+      <c r="M17" s="12" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="n"/>
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>8 items (5 diode types, 3 thyristor types)</t>
         </is>
       </c>
-      <c r="D14" s="15" t="n"/>
-      <c r="E14" s="16" t="n">
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="22" t="n">
         <v>857</v>
       </c>
-      <c r="F14" s="17" t="n">
+      <c r="F18" s="23" t="n">
         <v>394.1</v>
       </c>
-      <c r="G14" s="17" t="n">
+      <c r="G18" s="23" t="n">
         <v>319.7</v>
       </c>
-      <c r="H14" s="15" t="n"/>
-      <c r="I14" s="17" t="n">
+      <c r="H18" s="21" t="n"/>
+      <c r="I18" s="23" t="n">
         <v>159393</v>
       </c>
-      <c r="J14" s="14" t="n"/>
-      <c r="K14" s="14" t="n"/>
-      <c r="L14" s="15" t="inlineStr">
+      <c r="J18" s="20" t="n"/>
+      <c r="K18" s="20" t="n"/>
+      <c r="L18" s="21" t="inlineStr">
         <is>
           <t>FCA Prague</t>
         </is>
       </c>
-      <c r="M14" s="15" t="inlineStr">
+      <c r="M18" s="21" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>Consistency checks:</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Incoterms — CONSISTENT across all 16 documents: FCA Prague (minor text variants 'FCA Prague, CZ' / 'FCA  Prague', same term).</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Currency  — CONSISTENT across all invoices: EUR (each invoice also shown in CZK at 1 EUR = 24.25 CZK, informational only).</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Gross weight for DN 0923634362 (5STP2552L0025) is printed as 0 on the delivery note — likely a data error; net weight 87 kg. Please verify.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  • No 'preferenční věta' (preferential-origin declaration) found in any document. Goods origin CZ; export to Japan at 0% VAT.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Delivery-note numbers are given in the 092… form shown on the delivery notes; invoices list the same number without the leading zero.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A13:M13"/>
+    <mergeCell ref="A6:M6"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>